<commit_message>
Added Pricing of financial derivatives python files, submitted Interest rates curve first TP
</commit_message>
<xml_diff>
--- a/3A - SFA/Interest rates curve models/TP 1 - Bootstrap oblig.xlsx
+++ b/3A - SFA/Interest rates curve models/TP 1 - Bootstrap oblig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\Mon Drive\Supports formations\ENSAE - MCTI\2026\Ressources cours MCTI 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arnaud\Desktop\MyGit\3A - SFA\Interest rates curve models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648BCE7A-381B-4BA1-938F-082F07FC4A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B7018A7-98D1-4188-ACC5-AE3A134E90FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="15634" xr2:uid="{5DF6A02F-8863-468F-B425-BD068CC169A7}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{D9EE2336-3009-48B4-84ED-E5651A528A88}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -47,36 +46,31 @@
     <t>Prix</t>
   </si>
   <si>
-    <t>DF</t>
+    <t>Taux :</t>
   </si>
   <si>
-    <t>Taux ZC</t>
+    <t>DF actuariel :</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000%"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Aptos Narrow"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -89,7 +83,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -97,33 +91,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -149,39 +128,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -233,7 +212,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -344,6 +323,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -352,13 +338,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -423,100 +402,163 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC897242-C83B-48BA-B505-6AC0DD8C7BC3}">
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126934A9-C8CC-45B1-B84F-53937CD5A056}">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5.5</v>
+      </c>
+      <c r="C2">
+        <v>104.25</v>
+      </c>
+      <c r="E2">
+        <f>C2/(100+B2)</f>
+        <v>0.98815165876777256</v>
+      </c>
+      <c r="F2" s="1">
+        <f>(1/E2)^(1/A2) -1</f>
+        <v>1.1990407673860837E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3.2</v>
+      </c>
+      <c r="C3">
+        <v>102.73</v>
+      </c>
+      <c r="E3">
+        <f>(C3-B3*SUM($E$2:E2))/(100+B3)</f>
+        <v>0.96480537492192953</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F5" si="0">(1/E3)^(1/A3) -1</f>
+        <v>1.8075867111683852E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>4.8</v>
+      </c>
+      <c r="C4">
+        <v>107.47</v>
+      </c>
+      <c r="E4">
+        <f>(C4-B4*SUM($E$2:E3))/(100+B4)</f>
+        <v>0.93602868547986096</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>2.2280979859979899E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A2" s="1">
+      <c r="B5">
+        <v>6.7</v>
+      </c>
+      <c r="C5">
+        <v>114.16</v>
+      </c>
+      <c r="E5">
+        <f>(C5-B5*SUM($E$2:E4))/(100+B5)</f>
+        <v>0.88850792578785309</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>2.9993949294881084E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="C2" s="2">
-        <v>104.25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" s="1">
+      <c r="B8">
+        <v>4.8</v>
+      </c>
+      <c r="C8">
+        <f>B8*E2</f>
+        <v>4.7431279620853077</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
-        <v>3.2</v>
-      </c>
-      <c r="C3" s="2">
-        <v>102.73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A4" s="1">
+      <c r="B9">
+        <v>4.8</v>
+      </c>
+      <c r="C9">
+        <f>B9*E3</f>
+        <v>4.6310657996252615</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="C4" s="2">
+      <c r="B10">
+        <v>104.8</v>
+      </c>
+      <c r="C10">
+        <f>B10*E4</f>
+        <v>98.095806238289427</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <f>B11*E5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <f>SUM(C8:C11)</f>
         <v>107.47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="C5" s="2">
-        <v>114.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>